<commit_message>
Excel: Kontrollwerte ins Uebersichtsblatt
LibreOffice laeuft in dieser Umgebung nicht (auch ein Workbook mit einer
einzigen SUM-Formel laeuft ins Timeout), die Formeln haben deshalb keine
zwischengespeicherten Werte und werden erst beim Oeffnen in Excel gerechnet.
Damit die Zahlen auch in einer Vorschau sichtbar sind, stehen sie zusaetzlich
im Klartext unter der Tabelle.

Geprueft: Formelbereiche decken exakt die Datenzeilen 2-415 ab, die Kriterien
liefern dieselben Zahlen wie das Auszaehlen der Daten
(Golf 103, Tennis 99, Schwimmen 180, Reiten/Eishockey 32).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TwwqEWQuBChyKpCZxs9c38
</commit_message>
<xml_diff>
--- a/coachgrid/Vereine_Schweiz.xlsx
+++ b/coachgrid/Vereine_Schweiz.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -702,66 +702,66 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Spalte «Link geprüft»</t>
+          <t>Kontrollwerte Stand 28.07.2026 (die Formeln oben müssen dasselbe ergeben)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Link ok – Website wurde am 28.07.2026 angesteuert und hat geantwortet (HTTP 200/301).</t>
+          <t>Golf: 103 Einträge, 92 mit Telefon, 71 mit E-Mail, 94 Websites ok</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Prüfen – Server blockt automatische Aufrufe (403/406) oder antwortete nicht rechtzeitig; im Browser meist normal erreichbar.</t>
+          <t>Tennis: 99 Einträge, 33 mit Telefon, 21 mit E-Mail, 79 Websites ok</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Link tot – Adresse liefert 404 oder einen Serverfehler.</t>
+          <t>Schwimmen: 180 Einträge, 0 mit Telefon, 0 mit E-Mail, 157 Websites ok</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Reiten &amp; Eishockey: 32 Einträge, 29 mit Telefon, 12 mit E-Mail, 19 Websites ok</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Was diese Liste NICHT ist</t>
-        </is>
-      </c>
+      <c r="A17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Telefonnummern und Mailadressen stammen 1:1 aus der Quelle und wurden nicht nachtelefoniert.</t>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Spalte «Link geprüft»</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>OpenStreetMap ist nicht vollständig: Vereine ohne eigene Anlage fehlen dort häufig ganz.</t>
+          <t>Link ok – Website wurde am 28.07.2026 angesteuert und hat geantwortet (HTTP 200/301).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Bei Schwimmen publiziert Swiss Aquatics keine Telefonnummern – dort gibt es Website und Ort.</t>
+          <t>Prüfen – Server blockt automatische Aufrufe (403/406) oder antwortete nicht rechtzeitig; im Browser meist normal erreichbar.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Für eine lückenlose Liste pro Sportart braucht es die Verbandsverzeichnisse (Swiss Tennis, Swiss Golf, football.ch, stv-fsg.ch, sihf.ch).</t>
+          <t>Link tot – Adresse liefert 404 oder einen Serverfehler.</t>
         </is>
       </c>
     </row>
@@ -769,14 +769,52 @@
       <c r="A22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Die Spalte «Priorität» kommt aus der Marktanalyse (coachgrid/marktanalyse-vereine.md):</t>
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Was diese Liste NICHT ist</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Telefonnummern und Mailadressen stammen 1:1 aus der Quelle und wurden nicht nachtelefoniert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>OpenStreetMap ist nicht vollständig: Vereine ohne eigene Anlage fehlen dort häufig ganz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Bei Schwimmen publiziert Swiss Aquatics keine Telefonnummern – dort gibt es Website und Ort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Für eine lückenlose Liste pro Sportart braucht es die Verbandsverzeichnisse (Swiss Tennis, Swiss Golf, football.ch, stv-fsg.ch, sihf.ch).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Die Spalte «Priorität» kommt aus der Marktanalyse (coachgrid/marktanalyse-vereine.md):</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>A = eigene Anlage und angestelltes Personal, echtes Budget. B = eigene Anlage, kleines Budget.</t>
         </is>

</xml_diff>